<commit_message>
History in Pascal command line interpreter
</commit_message>
<xml_diff>
--- a/Manuals/R65 OS Memory Map.xlsx
+++ b/Manuals/R65 OS Memory Map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rricharz/Projects/R65/Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{328A43F9-EA39-094B-B8B1-EB4162236D44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139DFF9F-49EE-F343-A1DD-86247036D421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="984" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="515">
   <si>
     <t>zone</t>
   </si>
@@ -1626,6 +1626,12 @@
   </si>
   <si>
     <t>User/Pascal</t>
+  </si>
+  <si>
+    <t>Pascal command history</t>
+  </si>
+  <si>
+    <t>Pascal</t>
   </si>
 </sst>
 </file>
@@ -5824,9 +5830,11 @@
         <v>256</v>
       </c>
       <c r="D158" s="5" t="s">
-        <v>508</v>
-      </c>
-      <c r="E158" s="5"/>
+        <v>513</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>514</v>
+      </c>
       <c r="F158" s="5"/>
       <c r="G158" s="5"/>
       <c r="H158" s="5"/>

</xml_diff>

<commit_message>
Fixed memory map table (free space)
</commit_message>
<xml_diff>
--- a/Manuals/R65 OS Memory Map.xlsx
+++ b/Manuals/R65 OS Memory Map.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rricharz/Projects/R65/Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56689EC5-8A3F-E744-8418-4B1F379C048E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951F9DA6-1516-1244-A0FD-CD3F710316E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5600" yWindow="600" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5580" yWindow="600" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="memory map" sheetId="1" r:id="rId1"/>
     <sheet name="notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'memory map'!$A$1:$H$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'memory map'!$A$1:$H$159</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'memory map'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="990" uniqueCount="518">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="522">
   <si>
     <t>zone</t>
   </si>
@@ -1628,19 +1628,31 @@
     <t>Pascal</t>
   </si>
   <si>
-    <t>17d7-17fe</t>
-  </si>
-  <si>
     <t>17ff</t>
   </si>
   <si>
     <t>savs</t>
   </si>
   <si>
-    <t>free? 17f2/f3 used in firmware</t>
-  </si>
-  <si>
     <t>unknown</t>
+  </si>
+  <si>
+    <t>17e7-17ff</t>
+  </si>
+  <si>
+    <t>KIM-1</t>
+  </si>
+  <si>
+    <t>KIM-1 Data Aera</t>
+  </si>
+  <si>
+    <t>17f2/3 set by monitor</t>
+  </si>
+  <si>
+    <t>17d7-17e6</t>
+  </si>
+  <si>
+    <t>free after startup</t>
   </si>
 </sst>
 </file>
@@ -2012,7 +2024,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="9.5" style="4" customWidth="1"/>
@@ -5735,14 +5747,14 @@
         <v>506</v>
       </c>
       <c r="B153" s="8" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="C153" s="8"/>
       <c r="D153" s="8" t="s">
-        <v>516</v>
+        <v>78</v>
       </c>
       <c r="E153" s="12" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
       <c r="F153" s="12"/>
       <c r="G153" s="12"/>
@@ -5753,143 +5765,165 @@
         <v>506</v>
       </c>
       <c r="B154" s="8" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="C154" s="8"/>
       <c r="D154" s="8" t="s">
-        <v>515</v>
-      </c>
-      <c r="E154" s="8" t="s">
-        <v>512</v>
-      </c>
-      <c r="F154" s="8"/>
-      <c r="G154" s="8"/>
-      <c r="H154" s="8"/>
-    </row>
-    <row r="155" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1" thickBot="1">
-      <c r="A155" s="9" t="s">
-        <v>509</v>
+        <v>521</v>
+      </c>
+      <c r="E154" s="12" t="s">
+        <v>517</v>
+      </c>
+      <c r="F154" s="12" t="s">
+        <v>518</v>
+      </c>
+      <c r="G154" s="12" t="s">
+        <v>519</v>
+      </c>
+      <c r="H154" s="12"/>
+    </row>
+    <row r="155" spans="1:8" ht="32" customHeight="1" thickBot="1">
+      <c r="A155" s="7" t="s">
+        <v>506</v>
       </c>
       <c r="B155" s="8" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="C155" s="8"/>
       <c r="D155" s="8" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="E155" s="8" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F155" s="8"/>
       <c r="G155" s="8"/>
       <c r="H155" s="8"/>
     </row>
-    <row r="156" spans="1:8" ht="32" customHeight="1">
-      <c r="A156" s="11" t="s">
+    <row r="156" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1" thickBot="1">
+      <c r="A156" s="9" t="s">
+        <v>509</v>
+      </c>
+      <c r="B156" s="8" t="s">
+        <v>509</v>
+      </c>
+      <c r="C156" s="8"/>
+      <c r="D156" s="8" t="s">
+        <v>510</v>
+      </c>
+      <c r="E156" s="8" t="s">
+        <v>510</v>
+      </c>
+      <c r="F156" s="8"/>
+      <c r="G156" s="8"/>
+      <c r="H156" s="8"/>
+    </row>
+    <row r="157" spans="1:8" ht="32" customHeight="1">
+      <c r="A157" s="11" t="s">
         <v>507</v>
       </c>
-      <c r="B156" s="12" t="s">
+      <c r="B157" s="12" t="s">
         <v>507</v>
       </c>
-      <c r="C156" s="12"/>
-      <c r="D156" s="12" t="s">
+      <c r="C157" s="12"/>
+      <c r="D157" s="12" t="s">
         <v>508</v>
       </c>
-      <c r="E156" s="12"/>
-      <c r="F156" s="12"/>
-      <c r="G156" s="12"/>
-      <c r="H156" s="12"/>
-    </row>
-    <row r="157" spans="1:8" ht="32" customHeight="1">
-      <c r="A157" s="6" t="s">
+      <c r="E157" s="12"/>
+      <c r="F157" s="12"/>
+      <c r="G157" s="12"/>
+      <c r="H157" s="12"/>
+    </row>
+    <row r="158" spans="1:8" ht="32" customHeight="1">
+      <c r="A158" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="B157" s="6" t="s">
+      <c r="B158" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="C157" s="6">
+      <c r="C158" s="6">
         <v>256</v>
       </c>
-      <c r="D157" s="6" t="s">
+      <c r="D158" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="E157" s="6" t="s">
+      <c r="E158" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="F157" s="6" t="s">
+      <c r="F158" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="G157" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H157" s="6"/>
-    </row>
-    <row r="158" spans="1:8" ht="32" customHeight="1">
-      <c r="A158" s="5" t="s">
-        <v>501</v>
-      </c>
-      <c r="B158" s="5" t="s">
-        <v>484</v>
-      </c>
-      <c r="C158" s="5">
-        <v>2048</v>
-      </c>
-      <c r="D158" s="5" t="s">
-        <v>485</v>
-      </c>
-      <c r="E158" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="F158" s="5" t="s">
-        <v>486</v>
-      </c>
-      <c r="G158" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H158" s="5"/>
+      <c r="G158" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="H158" s="6"/>
     </row>
     <row r="159" spans="1:8" ht="32" customHeight="1">
       <c r="A159" s="5" t="s">
         <v>501</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>502</v>
+        <v>484</v>
       </c>
       <c r="C159" s="5">
+        <v>2048</v>
+      </c>
+      <c r="D159" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="E159" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="D159" s="5" t="s">
-        <v>511</v>
-      </c>
-      <c r="E159" s="5" t="s">
-        <v>512</v>
-      </c>
-      <c r="F159" s="5"/>
-      <c r="G159" s="5"/>
+      <c r="F159" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="G159" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="H159" s="5"/>
     </row>
     <row r="160" spans="1:8" ht="32" customHeight="1">
       <c r="A160" s="5" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C160" s="5">
-        <v>4096</v>
+        <v>256</v>
       </c>
       <c r="D160" s="5" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="F160" s="5"/>
       <c r="G160" s="5"/>
       <c r="H160" s="5"/>
     </row>
+    <row r="161" spans="1:8" ht="32" customHeight="1">
+      <c r="A161" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="B161" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="C161" s="5">
+        <v>4096</v>
+      </c>
+      <c r="D161" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="E161" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="F161" s="5"/>
+      <c r="G161" s="5"/>
+      <c r="H161" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H158" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H159" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
   <pageSetup paperSize="11" scale="94" fitToHeight="0" orientation="landscape"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
Improved break system at Pascal level
</commit_message>
<xml_diff>
--- a/Manuals/R65 OS Memory Map.xlsx
+++ b/Manuals/R65 OS Memory Map.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rricharz/Projects/R65/Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951F9DA6-1516-1244-A0FD-CD3F710316E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC754AC-B452-4444-BC5D-2D7B981457B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5580" yWindow="600" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5580" yWindow="620" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="memory map" sheetId="1" r:id="rId1"/>
     <sheet name="notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'memory map'!$A$1:$H$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'memory map'!$A$1:$H$160</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'memory map'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="0"/>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="996" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="526">
   <si>
     <t>zone</t>
   </si>
@@ -1637,9 +1637,6 @@
     <t>unknown</t>
   </si>
   <si>
-    <t>17e7-17ff</t>
-  </si>
-  <si>
     <t>KIM-1</t>
   </si>
   <si>
@@ -1649,10 +1646,25 @@
     <t>17f2/3 set by monitor</t>
   </si>
   <si>
-    <t>17d7-17e6</t>
-  </si>
-  <si>
     <t>free after startup</t>
+  </si>
+  <si>
+    <t>pascal</t>
+  </si>
+  <si>
+    <t>trace counter</t>
+  </si>
+  <si>
+    <t>17d7</t>
+  </si>
+  <si>
+    <t>17d8-17e6</t>
+  </si>
+  <si>
+    <t>17e7-17fe</t>
+  </si>
+  <si>
+    <t>trcnt</t>
   </si>
 </sst>
 </file>
@@ -1731,7 +1743,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1768,26 +1780,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="slantDashDot">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FF7A7266"/>
-      </top>
-      <bottom style="slantDashDot">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1811,22 +1803,22 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2024,7 +2016,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H161"/>
+  <dimension ref="A1:H162"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="9.5" style="4" customWidth="1"/>
@@ -5742,188 +5734,210 @@
         <v>89</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="32" customHeight="1" thickBot="1">
-      <c r="A153" s="7" t="s">
+    <row r="153" spans="1:8" ht="32" customHeight="1">
+      <c r="A153" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="B153" s="8" t="s">
+      <c r="B153" s="5" t="s">
+        <v>522</v>
+      </c>
+      <c r="C153" s="5">
+        <v>1</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>525</v>
+      </c>
+      <c r="E153" s="5" t="s">
         <v>520</v>
       </c>
-      <c r="C153" s="8"/>
-      <c r="D153" s="8" t="s">
+      <c r="F153" s="5" t="s">
+        <v>521</v>
+      </c>
+      <c r="G153" s="5"/>
+      <c r="H153" s="5"/>
+    </row>
+    <row r="154" spans="1:8" ht="32" customHeight="1">
+      <c r="A154" s="11" t="s">
+        <v>506</v>
+      </c>
+      <c r="B154" s="9" t="s">
+        <v>523</v>
+      </c>
+      <c r="C154" s="9"/>
+      <c r="D154" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E153" s="12" t="s">
+      <c r="E154" s="9" t="s">
         <v>515</v>
       </c>
-      <c r="F153" s="12"/>
-      <c r="G153" s="12"/>
-      <c r="H153" s="12"/>
-    </row>
-    <row r="154" spans="1:8" ht="32" customHeight="1" thickBot="1">
-      <c r="A154" s="7" t="s">
+      <c r="F154" s="9"/>
+      <c r="G154" s="9"/>
+      <c r="H154" s="9"/>
+    </row>
+    <row r="155" spans="1:8" ht="32" customHeight="1">
+      <c r="A155" s="10" t="s">
         <v>506</v>
       </c>
-      <c r="B154" s="8" t="s">
+      <c r="B155" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="C155" s="9"/>
+      <c r="D155" s="9" t="s">
+        <v>519</v>
+      </c>
+      <c r="E155" s="9" t="s">
         <v>516</v>
       </c>
-      <c r="C154" s="8"/>
-      <c r="D154" s="8" t="s">
-        <v>521</v>
-      </c>
-      <c r="E154" s="12" t="s">
+      <c r="F155" s="9" t="s">
         <v>517</v>
       </c>
-      <c r="F154" s="12" t="s">
+      <c r="G155" s="9" t="s">
         <v>518</v>
       </c>
-      <c r="G154" s="12" t="s">
-        <v>519</v>
-      </c>
-      <c r="H154" s="12"/>
-    </row>
-    <row r="155" spans="1:8" ht="32" customHeight="1" thickBot="1">
-      <c r="A155" s="7" t="s">
+      <c r="H155" s="9"/>
+    </row>
+    <row r="156" spans="1:8" s="12" customFormat="1" ht="32" customHeight="1">
+      <c r="A156" s="10" t="s">
         <v>506</v>
       </c>
-      <c r="B155" s="8" t="s">
+      <c r="B156" s="9" t="s">
         <v>513</v>
       </c>
-      <c r="C155" s="8"/>
-      <c r="D155" s="8" t="s">
+      <c r="C156" s="9"/>
+      <c r="D156" s="9" t="s">
         <v>514</v>
       </c>
-      <c r="E155" s="8" t="s">
+      <c r="E156" s="9" t="s">
         <v>512</v>
       </c>
-      <c r="F155" s="8"/>
-      <c r="G155" s="8"/>
-      <c r="H155" s="8"/>
-    </row>
-    <row r="156" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1" thickBot="1">
-      <c r="A156" s="9" t="s">
+      <c r="F156" s="9"/>
+      <c r="G156" s="9"/>
+      <c r="H156" s="9"/>
+    </row>
+    <row r="157" spans="1:8" s="12" customFormat="1" ht="32" customHeight="1">
+      <c r="A157" s="10" t="s">
         <v>509</v>
       </c>
-      <c r="B156" s="8" t="s">
+      <c r="B157" s="9" t="s">
         <v>509</v>
       </c>
-      <c r="C156" s="8"/>
-      <c r="D156" s="8" t="s">
+      <c r="C157" s="9"/>
+      <c r="D157" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="E156" s="8" t="s">
+      <c r="E157" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="F156" s="8"/>
-      <c r="G156" s="8"/>
-      <c r="H156" s="8"/>
-    </row>
-    <row r="157" spans="1:8" ht="32" customHeight="1">
-      <c r="A157" s="11" t="s">
+      <c r="F157" s="9"/>
+      <c r="G157" s="9"/>
+      <c r="H157" s="9"/>
+    </row>
+    <row r="158" spans="1:8" ht="32" customHeight="1">
+      <c r="A158" s="7" t="s">
         <v>507</v>
       </c>
-      <c r="B157" s="12" t="s">
+      <c r="B158" s="8" t="s">
         <v>507</v>
       </c>
-      <c r="C157" s="12"/>
-      <c r="D157" s="12" t="s">
+      <c r="C158" s="8"/>
+      <c r="D158" s="8" t="s">
         <v>508</v>
       </c>
-      <c r="E157" s="12"/>
-      <c r="F157" s="12"/>
-      <c r="G157" s="12"/>
-      <c r="H157" s="12"/>
-    </row>
-    <row r="158" spans="1:8" ht="32" customHeight="1">
-      <c r="A158" s="6" t="s">
+      <c r="E158" s="8"/>
+      <c r="F158" s="8"/>
+      <c r="G158" s="8"/>
+      <c r="H158" s="8"/>
+    </row>
+    <row r="159" spans="1:8" ht="32" customHeight="1">
+      <c r="A159" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="B158" s="6" t="s">
+      <c r="B159" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="C158" s="6">
+      <c r="C159" s="6">
         <v>256</v>
       </c>
-      <c r="D158" s="6" t="s">
+      <c r="D159" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="E158" s="6" t="s">
+      <c r="E159" s="6" t="s">
         <v>256</v>
       </c>
-      <c r="F158" s="6" t="s">
+      <c r="F159" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="G158" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H158" s="6"/>
-    </row>
-    <row r="159" spans="1:8" ht="32" customHeight="1">
-      <c r="A159" s="5" t="s">
-        <v>501</v>
-      </c>
-      <c r="B159" s="5" t="s">
-        <v>484</v>
-      </c>
-      <c r="C159" s="5">
-        <v>2048</v>
-      </c>
-      <c r="D159" s="5" t="s">
-        <v>485</v>
-      </c>
-      <c r="E159" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="F159" s="5" t="s">
-        <v>486</v>
-      </c>
-      <c r="G159" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="H159" s="5"/>
+      <c r="G159" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="H159" s="6"/>
     </row>
     <row r="160" spans="1:8" ht="32" customHeight="1">
       <c r="A160" s="5" t="s">
         <v>501</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>502</v>
+        <v>484</v>
       </c>
       <c r="C160" s="5">
+        <v>2048</v>
+      </c>
+      <c r="D160" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="E160" s="5" t="s">
         <v>256</v>
       </c>
-      <c r="D160" s="5" t="s">
-        <v>511</v>
-      </c>
-      <c r="E160" s="5" t="s">
-        <v>512</v>
-      </c>
-      <c r="F160" s="5"/>
-      <c r="G160" s="5"/>
+      <c r="F160" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="G160" s="5" t="s">
+        <v>88</v>
+      </c>
       <c r="H160" s="5"/>
     </row>
     <row r="161" spans="1:8" ht="32" customHeight="1">
       <c r="A161" s="5" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="C161" s="5">
-        <v>4096</v>
+        <v>256</v>
       </c>
       <c r="D161" s="5" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="E161" s="5" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="F161" s="5"/>
       <c r="G161" s="5"/>
       <c r="H161" s="5"/>
     </row>
+    <row r="162" spans="1:8" ht="32" customHeight="1">
+      <c r="A162" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="B162" s="5" t="s">
+        <v>503</v>
+      </c>
+      <c r="C162" s="5">
+        <v>4096</v>
+      </c>
+      <c r="D162" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="E162" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="F162" s="5"/>
+      <c r="G162" s="5"/>
+      <c r="H162" s="5"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H159" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H160" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
   <pageSetup paperSize="11" scale="94" fitToHeight="0" orientation="landscape"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>

<commit_message>
Continue with the deveopment of WRITELIB
</commit_message>
<xml_diff>
--- a/Manuals/R65 OS Memory Map.xlsx
+++ b/Manuals/R65 OS Memory Map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rricharz/Projects/R65/Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCC754AC-B452-4444-BC5D-2D7B981457B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A14B520-0F98-9A4C-8377-D469851606F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="620" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="524">
   <si>
     <t>zone</t>
   </si>
@@ -1634,21 +1634,9 @@
     <t>savs</t>
   </si>
   <si>
-    <t>unknown</t>
-  </si>
-  <si>
-    <t>KIM-1</t>
-  </si>
-  <si>
-    <t>KIM-1 Data Aera</t>
-  </si>
-  <si>
     <t>17f2/3 set by monitor</t>
   </si>
   <si>
-    <t>free after startup</t>
-  </si>
-  <si>
     <t>pascal</t>
   </si>
   <si>
@@ -1658,13 +1646,19 @@
     <t>17d7</t>
   </si>
   <si>
-    <t>17d8-17e6</t>
-  </si>
-  <si>
-    <t>17e7-17fe</t>
-  </si>
-  <si>
     <t>trcnt</t>
+  </si>
+  <si>
+    <t>writbuf</t>
+  </si>
+  <si>
+    <t>temporary buffer</t>
+  </si>
+  <si>
+    <t>17d8-17e8</t>
+  </si>
+  <si>
+    <t>17e9-17fe</t>
   </si>
 </sst>
 </file>
@@ -1743,7 +1737,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1780,12 +1774,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF7A7266"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="hair">
+        <color auto="1"/>
+      </top>
+      <bottom style="hair">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1803,22 +1828,26 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -5739,138 +5768,136 @@
         <v>506</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="C153" s="5">
         <v>1</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
       <c r="E153" s="5" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="F153" s="5" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="G153" s="5"/>
       <c r="H153" s="5"/>
     </row>
-    <row r="154" spans="1:8" ht="32" customHeight="1">
+    <row r="154" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1">
       <c r="A154" s="11" t="s">
         <v>506</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="C154" s="9"/>
       <c r="D154" s="9" t="s">
-        <v>78</v>
+        <v>520</v>
       </c>
       <c r="E154" s="9" t="s">
-        <v>515</v>
-      </c>
-      <c r="F154" s="9"/>
+        <v>512</v>
+      </c>
+      <c r="F154" s="9" t="s">
+        <v>521</v>
+      </c>
       <c r="G154" s="9"/>
       <c r="H154" s="9"/>
     </row>
-    <row r="155" spans="1:8" ht="32" customHeight="1">
-      <c r="A155" s="10" t="s">
+    <row r="155" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
+      <c r="A155" s="12" t="s">
         <v>506</v>
       </c>
-      <c r="B155" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="C155" s="9"/>
-      <c r="D155" s="9" t="s">
-        <v>519</v>
-      </c>
-      <c r="E155" s="9" t="s">
-        <v>516</v>
-      </c>
-      <c r="F155" s="9" t="s">
-        <v>517</v>
-      </c>
+      <c r="B155" s="13" t="s">
+        <v>523</v>
+      </c>
+      <c r="C155" s="13"/>
+      <c r="D155" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E155" s="13"/>
+      <c r="F155" s="13"/>
       <c r="G155" s="9" t="s">
-        <v>518</v>
-      </c>
-      <c r="H155" s="9"/>
-    </row>
-    <row r="156" spans="1:8" s="12" customFormat="1" ht="32" customHeight="1">
-      <c r="A156" s="10" t="s">
+        <v>515</v>
+      </c>
+      <c r="H155" s="13"/>
+    </row>
+    <row r="156" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
+      <c r="A156" s="12" t="s">
         <v>506</v>
       </c>
-      <c r="B156" s="9" t="s">
+      <c r="B156" s="13" t="s">
         <v>513</v>
       </c>
-      <c r="C156" s="9"/>
-      <c r="D156" s="9" t="s">
+      <c r="C156" s="13"/>
+      <c r="D156" s="13" t="s">
         <v>514</v>
       </c>
-      <c r="E156" s="9" t="s">
+      <c r="E156" s="13" t="s">
         <v>512</v>
       </c>
-      <c r="F156" s="9"/>
-      <c r="G156" s="9"/>
-      <c r="H156" s="9"/>
-    </row>
-    <row r="157" spans="1:8" s="12" customFormat="1" ht="32" customHeight="1">
-      <c r="A157" s="10" t="s">
+      <c r="F156" s="13"/>
+      <c r="G156" s="13"/>
+      <c r="H156" s="13"/>
+    </row>
+    <row r="157" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">
+      <c r="A157" s="12" t="s">
         <v>509</v>
       </c>
-      <c r="B157" s="9" t="s">
+      <c r="B157" s="13" t="s">
         <v>509</v>
       </c>
-      <c r="C157" s="9"/>
-      <c r="D157" s="9" t="s">
+      <c r="C157" s="13"/>
+      <c r="D157" s="13" t="s">
         <v>510</v>
       </c>
-      <c r="E157" s="9" t="s">
+      <c r="E157" s="13" t="s">
         <v>510</v>
       </c>
-      <c r="F157" s="9"/>
-      <c r="G157" s="9"/>
-      <c r="H157" s="9"/>
-    </row>
-    <row r="158" spans="1:8" ht="32" customHeight="1">
-      <c r="A158" s="7" t="s">
+      <c r="F157" s="13"/>
+      <c r="G157" s="13"/>
+      <c r="H157" s="13"/>
+    </row>
+    <row r="158" spans="1:8" s="10" customFormat="1" ht="32" customHeight="1">
+      <c r="A158" s="8" t="s">
         <v>507</v>
       </c>
-      <c r="B158" s="8" t="s">
+      <c r="B158" s="9" t="s">
         <v>507</v>
       </c>
-      <c r="C158" s="8"/>
-      <c r="D158" s="8" t="s">
+      <c r="C158" s="9"/>
+      <c r="D158" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="E158" s="8"/>
-      <c r="F158" s="8"/>
-      <c r="G158" s="8"/>
-      <c r="H158" s="8"/>
+      <c r="E158" s="9"/>
+      <c r="F158" s="9"/>
+      <c r="G158" s="9"/>
+      <c r="H158" s="9"/>
     </row>
     <row r="159" spans="1:8" ht="32" customHeight="1">
-      <c r="A159" s="6" t="s">
+      <c r="A159" s="7" t="s">
         <v>501</v>
       </c>
-      <c r="B159" s="6" t="s">
+      <c r="B159" s="7" t="s">
         <v>481</v>
       </c>
-      <c r="C159" s="6">
+      <c r="C159" s="7">
         <v>256</v>
       </c>
-      <c r="D159" s="6" t="s">
+      <c r="D159" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="E159" s="6" t="s">
+      <c r="E159" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="F159" s="6" t="s">
+      <c r="F159" s="7" t="s">
         <v>483</v>
       </c>
-      <c r="G159" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="H159" s="6"/>
+      <c r="G159" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="H159" s="7"/>
     </row>
     <row r="160" spans="1:8" ht="32" customHeight="1">
       <c r="A160" s="5" t="s">

</xml_diff>

<commit_message>
Fixed short constant strings, started work on FUNCTION
</commit_message>
<xml_diff>
--- a/Manuals/R65 OS Memory Map.xlsx
+++ b/Manuals/R65 OS Memory Map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rricharz/Projects/R65/Manuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A14B520-0F98-9A4C-8377-D469851606F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D99FC8C-4328-604B-962A-1E4C4161367E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5580" yWindow="620" windowWidth="19120" windowHeight="16760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="525">
   <si>
     <t>zone</t>
   </si>
@@ -1655,10 +1655,13 @@
     <t>temporary buffer</t>
   </si>
   <si>
-    <t>17d8-17e8</t>
-  </si>
-  <si>
-    <t>17e9-17fe</t>
+    <t>17d8-17f1</t>
+  </si>
+  <si>
+    <t>17f2-17fe</t>
+  </si>
+  <si>
+    <t>25 bytes</t>
   </si>
 </sst>
 </file>
@@ -1828,7 +1831,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5802,7 +5805,9 @@
       <c r="F154" s="9" t="s">
         <v>521</v>
       </c>
-      <c r="G154" s="9"/>
+      <c r="G154" s="9" t="s">
+        <v>524</v>
+      </c>
       <c r="H154" s="9"/>
     </row>
     <row r="155" spans="1:8" s="14" customFormat="1" ht="32" customHeight="1">

</xml_diff>